<commit_message>
update data files and fix output formatting in notebooks
</commit_message>
<xml_diff>
--- a/crude_oil_2025.xlsx
+++ b/crude_oil_2025.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F226"/>
+  <dimension ref="A1:F251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4942,7 +4942,7 @@
         <v>59.79999923706055</v>
       </c>
       <c r="F225" t="n">
-        <v>334116</v>
+        <v>189638</v>
       </c>
     </row>
     <row r="226">
@@ -4950,19 +4950,519 @@
         <v>45979</v>
       </c>
       <c r="B226" t="n">
-        <v>59.29999923706055</v>
+        <v>60.7400016784668</v>
       </c>
       <c r="C226" t="n">
-        <v>59.86000061035156</v>
+        <v>60.93000030517578</v>
       </c>
       <c r="D226" t="n">
-        <v>59.33000183105469</v>
+        <v>59.31000137329102</v>
       </c>
       <c r="E226" t="n">
         <v>59.7400016784668</v>
       </c>
       <c r="F226" t="n">
-        <v>14574</v>
+        <v>105325</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>45980</v>
+      </c>
+      <c r="B227" t="n">
+        <v>59.43999862670898</v>
+      </c>
+      <c r="C227" t="n">
+        <v>60.79000091552734</v>
+      </c>
+      <c r="D227" t="n">
+        <v>58.77000045776367</v>
+      </c>
+      <c r="E227" t="n">
+        <v>60.61999893188477</v>
+      </c>
+      <c r="F227" t="n">
+        <v>79622</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B228" t="n">
+        <v>59.13999938964844</v>
+      </c>
+      <c r="C228" t="n">
+        <v>60.33000183105469</v>
+      </c>
+      <c r="D228" t="n">
+        <v>58.86000061035156</v>
+      </c>
+      <c r="E228" t="n">
+        <v>59.63000106811523</v>
+      </c>
+      <c r="F228" t="n">
+        <v>324282</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B229" t="n">
+        <v>58.06000137329102</v>
+      </c>
+      <c r="C229" t="n">
+        <v>58.79999923706055</v>
+      </c>
+      <c r="D229" t="n">
+        <v>57.38000106811523</v>
+      </c>
+      <c r="E229" t="n">
+        <v>58.79999923706055</v>
+      </c>
+      <c r="F229" t="n">
+        <v>345014</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B230" t="n">
+        <v>58.84000015258789</v>
+      </c>
+      <c r="C230" t="n">
+        <v>59.06000137329102</v>
+      </c>
+      <c r="D230" t="n">
+        <v>57.41999816894531</v>
+      </c>
+      <c r="E230" t="n">
+        <v>58.04999923706055</v>
+      </c>
+      <c r="F230" t="n">
+        <v>238138</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>45986</v>
+      </c>
+      <c r="B231" t="n">
+        <v>57.95000076293945</v>
+      </c>
+      <c r="C231" t="n">
+        <v>58.95999908447266</v>
+      </c>
+      <c r="D231" t="n">
+        <v>57.09999847412109</v>
+      </c>
+      <c r="E231" t="n">
+        <v>58.88999938964844</v>
+      </c>
+      <c r="F231" t="n">
+        <v>334442</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>45987</v>
+      </c>
+      <c r="B232" t="n">
+        <v>58.65000152587891</v>
+      </c>
+      <c r="C232" t="n">
+        <v>58.72000122070312</v>
+      </c>
+      <c r="D232" t="n">
+        <v>57.65999984741211</v>
+      </c>
+      <c r="E232" t="n">
+        <v>58.04999923706055</v>
+      </c>
+      <c r="F232" t="n">
+        <v>228285</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B233" t="n">
+        <v>58.54999923706055</v>
+      </c>
+      <c r="C233" t="n">
+        <v>59.63999938964844</v>
+      </c>
+      <c r="D233" t="n">
+        <v>58.27000045776367</v>
+      </c>
+      <c r="E233" t="n">
+        <v>58.58000183105469</v>
+      </c>
+      <c r="F233" t="n">
+        <v>153758</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B234" t="n">
+        <v>59.31999969482422</v>
+      </c>
+      <c r="C234" t="n">
+        <v>59.97000122070312</v>
+      </c>
+      <c r="D234" t="n">
+        <v>58.83000183105469</v>
+      </c>
+      <c r="E234" t="n">
+        <v>58.95999908447266</v>
+      </c>
+      <c r="F234" t="n">
+        <v>232770</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>45993</v>
+      </c>
+      <c r="B235" t="n">
+        <v>58.63999938964844</v>
+      </c>
+      <c r="C235" t="n">
+        <v>59.66999816894531</v>
+      </c>
+      <c r="D235" t="n">
+        <v>58.27999877929688</v>
+      </c>
+      <c r="E235" t="n">
+        <v>59.52000045776367</v>
+      </c>
+      <c r="F235" t="n">
+        <v>255513</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>45994</v>
+      </c>
+      <c r="B236" t="n">
+        <v>58.95000076293945</v>
+      </c>
+      <c r="C236" t="n">
+        <v>59.63999938964844</v>
+      </c>
+      <c r="D236" t="n">
+        <v>58.36999893188477</v>
+      </c>
+      <c r="E236" t="n">
+        <v>58.65000152587891</v>
+      </c>
+      <c r="F236" t="n">
+        <v>260974</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>45995</v>
+      </c>
+      <c r="B237" t="n">
+        <v>59.66999816894531</v>
+      </c>
+      <c r="C237" t="n">
+        <v>60.02000045776367</v>
+      </c>
+      <c r="D237" t="n">
+        <v>58.81000137329102</v>
+      </c>
+      <c r="E237" t="n">
+        <v>59.09000015258789</v>
+      </c>
+      <c r="F237" t="n">
+        <v>264993</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>45996</v>
+      </c>
+      <c r="B238" t="n">
+        <v>60.08000183105469</v>
+      </c>
+      <c r="C238" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="D238" t="n">
+        <v>59.41999816894531</v>
+      </c>
+      <c r="E238" t="n">
+        <v>59.70000076293945</v>
+      </c>
+      <c r="F238" t="n">
+        <v>255075</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B239" t="n">
+        <v>58.88000106811523</v>
+      </c>
+      <c r="C239" t="n">
+        <v>60.29999923706055</v>
+      </c>
+      <c r="D239" t="n">
+        <v>58.68000030517578</v>
+      </c>
+      <c r="E239" t="n">
+        <v>60.15000152587891</v>
+      </c>
+      <c r="F239" t="n">
+        <v>263009</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46000</v>
+      </c>
+      <c r="B240" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="C240" t="n">
+        <v>59.16999816894531</v>
+      </c>
+      <c r="D240" t="n">
+        <v>58.11999893188477</v>
+      </c>
+      <c r="E240" t="n">
+        <v>58.86999893188477</v>
+      </c>
+      <c r="F240" t="n">
+        <v>260206</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46001</v>
+      </c>
+      <c r="B241" t="n">
+        <v>58.45999908447266</v>
+      </c>
+      <c r="C241" t="n">
+        <v>59.04999923706055</v>
+      </c>
+      <c r="D241" t="n">
+        <v>57.65999984741211</v>
+      </c>
+      <c r="E241" t="n">
+        <v>58.36999893188477</v>
+      </c>
+      <c r="F241" t="n">
+        <v>256508</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46002</v>
+      </c>
+      <c r="B242" t="n">
+        <v>57.59999847412109</v>
+      </c>
+      <c r="C242" t="n">
+        <v>58.93999862670898</v>
+      </c>
+      <c r="D242" t="n">
+        <v>57.0099983215332</v>
+      </c>
+      <c r="E242" t="n">
+        <v>58.90999984741211</v>
+      </c>
+      <c r="F242" t="n">
+        <v>286808</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46003</v>
+      </c>
+      <c r="B243" t="n">
+        <v>57.43999862670898</v>
+      </c>
+      <c r="C243" t="n">
+        <v>58.18999862670898</v>
+      </c>
+      <c r="D243" t="n">
+        <v>57.15000152587891</v>
+      </c>
+      <c r="E243" t="n">
+        <v>57.88999938964844</v>
+      </c>
+      <c r="F243" t="n">
+        <v>212806</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B244" t="n">
+        <v>56.81999969482422</v>
+      </c>
+      <c r="C244" t="n">
+        <v>57.79999923706055</v>
+      </c>
+      <c r="D244" t="n">
+        <v>56.40000152587891</v>
+      </c>
+      <c r="E244" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="F244" t="n">
+        <v>229310</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B245" t="n">
+        <v>55.27000045776367</v>
+      </c>
+      <c r="C245" t="n">
+        <v>56.70000076293945</v>
+      </c>
+      <c r="D245" t="n">
+        <v>54.97999954223633</v>
+      </c>
+      <c r="E245" t="n">
+        <v>56.68000030517578</v>
+      </c>
+      <c r="F245" t="n">
+        <v>230933</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B246" t="n">
+        <v>55.93999862670898</v>
+      </c>
+      <c r="C246" t="n">
+        <v>56.97999954223633</v>
+      </c>
+      <c r="D246" t="n">
+        <v>55.20000076293945</v>
+      </c>
+      <c r="E246" t="n">
+        <v>55.22999954223633</v>
+      </c>
+      <c r="F246" t="n">
+        <v>125608</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B247" t="n">
+        <v>56.15000152587891</v>
+      </c>
+      <c r="C247" t="n">
+        <v>57.02999877929688</v>
+      </c>
+      <c r="D247" t="n">
+        <v>55.88000106811523</v>
+      </c>
+      <c r="E247" t="n">
+        <v>56.90000152587891</v>
+      </c>
+      <c r="F247" t="n">
+        <v>85735</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46010</v>
+      </c>
+      <c r="B248" t="n">
+        <v>56.65999984741211</v>
+      </c>
+      <c r="C248" t="n">
+        <v>56.90000152587891</v>
+      </c>
+      <c r="D248" t="n">
+        <v>55.81999969482422</v>
+      </c>
+      <c r="E248" t="n">
+        <v>56.02999877929688</v>
+      </c>
+      <c r="F248" t="n">
+        <v>209264</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B249" t="n">
+        <v>58.0099983215332</v>
+      </c>
+      <c r="C249" t="n">
+        <v>58.13000106811523</v>
+      </c>
+      <c r="D249" t="n">
+        <v>56.59999847412109</v>
+      </c>
+      <c r="E249" t="n">
+        <v>56.63000106811523</v>
+      </c>
+      <c r="F249" t="n">
+        <v>221576</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="B250" t="n">
+        <v>58.38000106811523</v>
+      </c>
+      <c r="C250" t="n">
+        <v>58.56000137329102</v>
+      </c>
+      <c r="D250" t="n">
+        <v>57.7400016784668</v>
+      </c>
+      <c r="E250" t="n">
+        <v>57.95000076293945</v>
+      </c>
+      <c r="F250" t="n">
+        <v>183633</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46015</v>
+      </c>
+      <c r="B251" t="n">
+        <v>58.34999847412109</v>
+      </c>
+      <c r="C251" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="D251" t="n">
+        <v>58.13000106811523</v>
+      </c>
+      <c r="E251" t="n">
+        <v>58.47000122070312</v>
+      </c>
+      <c r="F251" t="n">
+        <v>183633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>